<commit_message>
starting to swap out bart code
</commit_message>
<xml_diff>
--- a/artf3_complex12_summary.xlsx
+++ b/artf3_complex12_summary.xlsx
@@ -503,19 +503,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-0.001320256464172841</v>
+        <v>0.02468158642584068</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.003925346433338689</v>
+        <v>0.04316843969508225</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.008477443565989045</v>
+        <v>0.0482085034030588</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.006963415443145916</v>
+        <v>0.04781990611878175</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.005027011551630719</v>
+        <v>0.04226867117883617</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -532,19 +532,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.009245518538962435</v>
+        <v>0.03683986575645156</v>
       </c>
       <c r="E3" t="n">
-        <v>0.005555970195021598</v>
+        <v>0.05290863338836135</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.006386957028549908</v>
+        <v>0.06135465294236086</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.01875753290064492</v>
+        <v>0.06004727225701503</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.02006865630928848</v>
+        <v>0.04846153114668998</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -561,19 +561,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.005736175122486788</v>
+        <v>0.03769370931962444</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0003849189183798153</v>
+        <v>0.05504188099751715</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.01215931510082387</v>
+        <v>0.06112148916245677</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.01980634327642085</v>
+        <v>0.0612839537889879</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.01790388149616239</v>
+        <v>0.04991695815066307</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -875,19 +875,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.01443122844383238</v>
+        <v>0.008792650290163588</v>
       </c>
       <c r="E14" t="n">
-        <v>0.02016704880779242</v>
+        <v>0.01229508716954023</v>
       </c>
       <c r="F14" t="n">
-        <v>0.02060715414366761</v>
+        <v>0.012088097398858</v>
       </c>
       <c r="G14" t="n">
-        <v>0.02137717675820465</v>
+        <v>0.01392566802996906</v>
       </c>
       <c r="H14" t="n">
-        <v>0.01731338005448291</v>
+        <v>0.01200600523312727</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -904,19 +904,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.01423687957921386</v>
+        <v>0.01054361018613424</v>
       </c>
       <c r="E15" t="n">
-        <v>0.01933138203479869</v>
+        <v>0.01142657428792278</v>
       </c>
       <c r="F15" t="n">
-        <v>0.01970321581340575</v>
+        <v>0.01309881887200237</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01924549907826907</v>
+        <v>0.01102396085430059</v>
       </c>
       <c r="H15" t="n">
-        <v>0.01437357305141341</v>
+        <v>0.01264990613867699</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -933,19 +933,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.01438641140528822</v>
+        <v>0.0106758309210167</v>
       </c>
       <c r="E16" t="n">
-        <v>0.01982731264895657</v>
+        <v>0.01191501892643991</v>
       </c>
       <c r="F16" t="n">
-        <v>0.02081140366782585</v>
+        <v>0.01275700393275258</v>
       </c>
       <c r="G16" t="n">
-        <v>0.02130626470162031</v>
+        <v>0.01282210756988659</v>
       </c>
       <c r="H16" t="n">
-        <v>0.01643050338687601</v>
+        <v>0.01398440932483678</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         <v>0.008539292742253648</v>
       </c>
       <c r="E25" t="n">
-        <v>0.01183583888984514</v>
+        <v>0.01183583888984515</v>
       </c>
       <c r="F25" t="n">
         <v>0.01542536864637076</v>
@@ -1247,19 +1247,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-0.001879229889851018</v>
+        <v>0.02330679439284319</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.002256337108057595</v>
+        <v>0.04163598119984087</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.009752074336643381</v>
+        <v>0.04679942959813232</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.006571682182789761</v>
+        <v>0.04674977906803827</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.005018256986151572</v>
+        <v>0.04117445670222777</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1276,19 +1276,19 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.00892369410927223</v>
+        <v>0.03530951303231365</v>
       </c>
       <c r="E27" t="n">
-        <v>0.00674166575469911</v>
+        <v>0.05145895687977913</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.0077662537032801</v>
+        <v>0.05964366799306528</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.01813212608212748</v>
+        <v>0.05857728516096295</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.01994739183229395</v>
+        <v>0.04666353245515235</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1305,19 +1305,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.00530395861844488</v>
+        <v>0.03646938437592241</v>
       </c>
       <c r="E28" t="n">
-        <v>0.001972497568961892</v>
+        <v>0.05296555740729653</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.01287095300831288</v>
+        <v>0.05991343801658594</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.01905779145395656</v>
+        <v>0.06050195834506836</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.01826185487721748</v>
+        <v>0.04791650874815022</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1619,19 +1619,19 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-0.01121330871240689</v>
+        <v>0.01841451385093976</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.01667575027488983</v>
+        <v>0.03467143230445192</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.0205518847283544</v>
+        <v>0.03994942388951767</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.02182894691830438</v>
+        <v>0.03777825659251279</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.01801554747013183</v>
+        <v>0.03346700310335578</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1648,19 +1648,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-0.0008014792292615735</v>
+        <v>0.0294629373065569</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.008467229157126631</v>
+        <v>0.04500954688873054</v>
       </c>
       <c r="F39" t="n">
-        <v>-0.02008512658557897</v>
+        <v>0.0517619186020843</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.03260512761455722</v>
+        <v>0.0524075606094817</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.02990435720527615</v>
+        <v>0.03884671741189365</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -1677,19 +1677,19 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-0.003950738321500454</v>
+        <v>0.02961576381702091</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.01372933602663665</v>
+        <v>0.04714106252181934</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.02632838722782419</v>
+        <v>0.05289201525727193</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0348644608026609</v>
+        <v>0.05199093869512027</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.02867515274491944</v>
+        <v>0.04033252564008377</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1991,19 +1991,19 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.007197763887243576</v>
+        <v>0.02901952285446032</v>
       </c>
       <c r="E50" t="n">
-        <v>0.009305545588062847</v>
+        <v>0.05121971132089347</v>
       </c>
       <c r="F50" t="n">
-        <v>0.005415391375791515</v>
+        <v>0.05529644120756489</v>
       </c>
       <c r="G50" t="n">
-        <v>0.006198149321896131</v>
+        <v>0.05525509374758292</v>
       </c>
       <c r="H50" t="n">
-        <v>0.007139688029681992</v>
+        <v>0.04920385681670551</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2020,19 +2020,19 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.01815224643884091</v>
+        <v>0.04135052564310858</v>
       </c>
       <c r="E51" t="n">
-        <v>0.01869911310972381</v>
+        <v>0.06111200650089044</v>
       </c>
       <c r="F51" t="n">
-        <v>0.005223108691758635</v>
+        <v>0.06956694003116573</v>
       </c>
       <c r="G51" t="n">
-        <v>-0.006024956599740087</v>
+        <v>0.06686121883783559</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.009564438723685006</v>
+        <v>0.05689603821094655</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2049,19 +2049,19 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.01430605080255094</v>
+        <v>0.04214343043536776</v>
       </c>
       <c r="E52" t="n">
-        <v>0.01377665097308001</v>
+        <v>0.06314783715077327</v>
       </c>
       <c r="F52" t="n">
-        <v>8.224502933161103e-05</v>
+        <v>0.06792473593098369</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.008786649948949897</v>
+        <v>0.06902849516575588</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.004794896650824296</v>
+        <v>0.0584237990446535</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>

</xml_diff>